<commit_message>
Add search block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 8
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-search.report.xlsx
+++ b/tools/importer/reports/import-search.report.xlsx
@@ -73,7 +73,7 @@
     <t>us/en/ent/search.report.json</t>
   </si>
   <si>
-    <t>[]</t>
+    <t>["search"]</t>
   </si>
   <si>
     <t>us/en/ent/search</t>
@@ -82,7 +82,7 @@
     <t>search</t>
   </si>
   <si>
-    <t>2026-10-12T11:03:20.778Z</t>
+    <t>2026-10-12T11:38:46.522Z</t>
   </si>
   <si>
     <t>Search | Stryker</t>

</xml_diff>